<commit_message>
css değişikliklerine devam edildi
</commit_message>
<xml_diff>
--- a/WebApplication11/Temp/ornek-stok-listesi (1).xlsx
+++ b/WebApplication11/Temp/ornek-stok-listesi (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kackinmuharrem\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80904285-8883-4B2F-95AD-52B4F67172E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B5B0467-F561-4236-A812-9F1CB070313B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -442,10 +442,10 @@
   <cols>
     <col min="1" max="1" width="10.140625" customWidth="1"/>
     <col min="2" max="3" width="11.85546875" customWidth="1"/>
-    <col min="4" max="4" width="9" customWidth="1"/>
-    <col min="5" max="5" width="17.7109375" customWidth="1"/>
-    <col min="6" max="6" width="9" customWidth="1"/>
-    <col min="7" max="7" width="12.5703125" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" customWidth="1"/>
+    <col min="5" max="5" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11" customWidth="1"/>
     <col min="9" max="9" width="12.42578125" customWidth="1"/>
     <col min="10" max="10" width="8.5703125" customWidth="1"/>
@@ -485,22 +485,22 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>9</v>
@@ -552,23 +552,23 @@
       <c r="C2" t="s">
         <v>27</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2">
+        <v>1.2</v>
+      </c>
+      <c r="H2">
+        <v>1.2</v>
+      </c>
+      <c r="I2">
         <v>1.1000000000000001</v>
-      </c>
-      <c r="E2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H2">
-        <v>1.2</v>
-      </c>
-      <c r="I2">
-        <v>1.2</v>
       </c>
       <c r="J2">
         <v>1.2</v>

</xml_diff>